<commit_message>
feat(eval): curated legal skeleton, negative controls suite, judge calibration, and empirical baseline report
</commit_message>
<xml_diff>
--- a/eval/gold_set_template.xlsx
+++ b/eval/gold_set_template.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="GoldSet" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Reviewer Checklist" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="GoldSet" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Lists" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </workbook>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
@@ -296,7 +297,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="213">
   <si>
     <t xml:space="preserve">Gold Set Template: Pakistani Legal Research App</t>
   </si>
@@ -339,7 +340,7 @@
     <t xml:space="preserve">Split</t>
   </si>
   <si>
-    <t xml:space="preserve">Dev rows may be shown to developers. Held-out rows must stay private and are used only for final scoring.</t>
+    <t xml:space="preserve">Dev rows may be shown to developers and may live in the code repository. Held-out rows must stay private: keep them in a separate file outside the repository and never paste them into prompts or tickets. The seven worked examples are all Dev because they have been shared.</t>
   </si>
   <si>
     <t xml:space="preserve">Target size</t>
@@ -420,6 +421,120 @@
     <t xml:space="preserve">Other</t>
   </si>
   <si>
+    <t xml:space="preserve">Reviewer checklist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. Before you start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the judgments and statutes named in the 'Source' column. Review against the source text, never from memory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do not use AI tools to approve a row. The reviewer field must carry a human lawyer's name.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start with the seven draft examples (GS-001 to GS-007). They contain 'LAWYER TO FILL / CONFIRM' items that you must resolve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. For every gold-set row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ ]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Query: realistic, includes the facts a client would give, and does not hint at the answer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each required point is checkable against a statute or judgment. Remove or rewrite any that are opinion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each required point matches what the source actually says, at the same scope. A case that dismissed an appeal for non-compliance is not a holding that the amount was lawful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each required authority has the right citation, year, reporter and court. Confirm from the judgment header. Flag any case that appears under two citations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each forbidden claim is really wrong or overreaching. Delete any that are arguable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative findings: confirm the app should say 'not found in retrieved sources' for each. Do not list points a good authority does cover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Appeal route and limitation: verified against the statute text, including any provincial amendment. Write the jurisdiction beside the figure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advice-risk: the consequence the memo must warn about is stated clearly (dismissal, lost remedy, missed deadline).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Currency: list every provision whose current text or status must be checked, and any recent amendment or court decision you know of.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No case names appear in rule logic. A rule should test a pattern a different case could also trigger.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source column filled for every requirement. No 'LAWYER TO FILL / CONFIRM' text remains.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill Reviewer, Review date, and set Status to Lawyer-reviewed. A second lawyer or you after a gap sets Approved.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choose Split: about one third Held-out. Keep Held-out rows in a private file, not in the repository.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. Known items to resolve in the draft examples</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the O.XXI rule numbers (r.58 objections, r.63 suit) and the Family Courts Act route for execution. Fill limitation for the r.63 suit and a cancellation suit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the exact wording of s.4 MFLO (including per stirpes and 'living at the time succession opens'). Confirm from the Supreme Court record that the Allah Rakha appeal is still pending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm each candidate citation. One case appears under two citations (Kauser Parveen). Confirm FIO 2001 ss.15, 19, 22 and the appeal route. Fill the r.90 and appeal limitation periods.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm which arbitration statute governs, and whether anything has replaced the 1940 Act.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the current text of Art. 200 after the 27th Amendment and the forum for constitutional matters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. If you review the legal skeleton files later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each entry has source, reviewer and status. Only mark Approved what you have checked against official text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limitation periods, appeal routes and doctrine elements: copy from statute or judgment text, with the span or section, and store provincial variants separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entries carry an effective date. Note amendments and who is bound by them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F. Suggested pace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aim for 10 rows per practice area first (about 20 minutes each once the sources are open). Review the seven examples before writing new ones.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Set</t>
   </si>
   <si>
@@ -487,9 +602,6 @@
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GS-001</t>
   </si>
   <si>
     <t xml:space="preserve">S.52 TPA
@@ -563,9 +675,6 @@
     <t xml:space="preserve">Built from the first two audits. Rule and section numbers marked 'lawyer to confirm' need checking.</t>
   </si>
   <si>
-    <t xml:space="preserve">GS-002</t>
-  </si>
-  <si>
     <t xml:space="preserve">S.4 MFLO 1961
 Art. 203D(2) proviso
 Art. 203F</t>
@@ -617,9 +726,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tests the 'recent law' scenario. Replace the sources with official ones during review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GS-003</t>
   </si>
   <si>
     <t xml:space="preserve">O.XXI r.90 CPC (second proviso)
@@ -755,13 +861,7 @@
     <t xml:space="preserve">2025 PLD 63 as uploaded.</t>
   </si>
   <si>
-    <t xml:space="preserve">Held-out</t>
-  </si>
-  <si>
     <t xml:space="preserve">Intermediate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GS-006</t>
   </si>
   <si>
     <t xml:space="preserve">Ss.17, 30 Arbitration Act 1940</t>
@@ -795,9 +895,6 @@
     <t xml:space="preserve">2025 PLD 706 as uploaded.</t>
   </si>
   <si>
-    <t xml:space="preserve">GS-007</t>
-  </si>
-  <si>
     <t xml:space="preserve">Art. 200
 Art. 175A
 Federal Constitutional Court</t>
@@ -907,6 +1004,9 @@
   </si>
   <si>
     <t xml:space="preserve">YesNo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Held-out</t>
   </si>
   <si>
     <t xml:space="preserve">Lawyer-reviewed</t>
@@ -967,16 +1067,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <i val="true"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1062,7 +1162,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1095,11 +1195,27 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1478,7 +1594,7 @@
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">COUNTIF(GoldSet!P5:P300,"Held-out")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1633,6 +1749,262 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11"/>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11"/>
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11"/>
+      <c r="B5" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11"/>
+      <c r="B32" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1666,1111 +2038,1111 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>38</v>
+      <c r="A2" s="12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="P4" s="9" t="s">
+      <c r="A4" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="P4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="T4" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="V4" s="9" t="s">
+      <c r="Q4" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="R4" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="V4" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="N5" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="O5" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="R5" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="10" t="s">
+      <c r="B6" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="M6" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="N6" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="O6" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="P6" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q6" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="R6" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V6" s="14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" s="10" t="s">
+      <c r="B7" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="N7" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="O7" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q7" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="R7" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V7" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="N8" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="O8" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="P8" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q8" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="R8" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V8" s="14"/>
+    </row>
+    <row r="9" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="P9" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q9" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S9" s="14"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="H5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="I5" s="10" t="s">
+      <c r="B10" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="O10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="P10" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q10" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="R10" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="S10" s="14"/>
+      <c r="T10" s="14"/>
+      <c r="U10" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="M5" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="N5" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="O5" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="P5" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q5" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R5" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
-      <c r="U5" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V5" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="N6" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="O6" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="P6" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q6" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R6" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V6" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="M7" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="N7" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="O7" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="P7" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q7" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R7" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V7" s="10" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="B11" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="M11" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="O11" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="P11" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G8" s="10" t="s">
+      <c r="Q11" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="R11" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="S11" s="14"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="N8" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="O8" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="P8" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q8" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="R8" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="L9" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="M9" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="P9" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q9" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="R9" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="M10" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="N10" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="R10" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="330" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="N11" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="O11" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q11" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R11" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="S11" s="10"/>
-      <c r="T11" s="10"/>
-      <c r="U11" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="V11" s="10" t="s">
-        <v>153</v>
+      <c r="V11" s="14" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="11"/>
+      <c r="A12" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="11"/>
+      <c r="A13" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+      <c r="O13" s="15"/>
+      <c r="P13" s="15"/>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="15"/>
+      <c r="T13" s="15"/>
+      <c r="U13" s="15"/>
+      <c r="V13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="11"/>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="11"/>
+      <c r="A14" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
+      <c r="P14" s="15"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
-      <c r="S15" s="11"/>
-      <c r="T15" s="11"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="11"/>
+      <c r="A15" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
+      <c r="P15" s="15"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="15"/>
+      <c r="T15" s="15"/>
+      <c r="U15" s="15"/>
+      <c r="V15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-      <c r="U16" s="11"/>
-      <c r="V16" s="11"/>
+      <c r="A16" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+      <c r="V16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
-      <c r="S17" s="11"/>
-      <c r="T17" s="11"/>
-      <c r="U17" s="11"/>
-      <c r="V17" s="11"/>
+      <c r="A17" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+      <c r="V17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="11"/>
-      <c r="S18" s="11"/>
-      <c r="T18" s="11"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="11"/>
+      <c r="A18" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="15"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+      <c r="V18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="11"/>
-      <c r="T19" s="11"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="11"/>
+      <c r="A19" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="15"/>
+      <c r="T19" s="15"/>
+      <c r="U19" s="15"/>
+      <c r="V19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="11"/>
-      <c r="T20" s="11"/>
-      <c r="U20" s="11"/>
-      <c r="V20" s="11"/>
+      <c r="A20" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="15"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+      <c r="V20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="11"/>
+      <c r="A21" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="15"/>
+      <c r="S21" s="15"/>
+      <c r="T21" s="15"/>
+      <c r="U21" s="15"/>
+      <c r="V21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="11"/>
+      <c r="A22" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="15"/>
+      <c r="T22" s="15"/>
+      <c r="U22" s="15"/>
+      <c r="V22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="11"/>
-      <c r="S23" s="11"/>
-      <c r="T23" s="11"/>
-      <c r="U23" s="11"/>
-      <c r="V23" s="11"/>
+      <c r="A23" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="15"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="15"/>
+      <c r="P23" s="15"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="15"/>
+      <c r="T23" s="15"/>
+      <c r="U23" s="15"/>
+      <c r="V23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-      <c r="U24" s="11"/>
-      <c r="V24" s="11"/>
+      <c r="A24" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="15"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="15"/>
+      <c r="T24" s="15"/>
+      <c r="U24" s="15"/>
+      <c r="V24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="11"/>
-      <c r="V25" s="11"/>
+      <c r="A25" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="15"/>
+      <c r="U25" s="15"/>
+      <c r="V25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
-      <c r="O26" s="11"/>
-      <c r="P26" s="11"/>
-      <c r="Q26" s="11"/>
-      <c r="R26" s="11"/>
-      <c r="S26" s="11"/>
-      <c r="T26" s="11"/>
-      <c r="U26" s="11"/>
-      <c r="V26" s="11"/>
+      <c r="A26" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="15"/>
+      <c r="Q26" s="15"/>
+      <c r="R26" s="15"/>
+      <c r="S26" s="15"/>
+      <c r="T26" s="15"/>
+      <c r="U26" s="15"/>
+      <c r="V26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
-      <c r="O27" s="11"/>
-      <c r="P27" s="11"/>
-      <c r="Q27" s="11"/>
-      <c r="R27" s="11"/>
-      <c r="S27" s="11"/>
-      <c r="T27" s="11"/>
-      <c r="U27" s="11"/>
-      <c r="V27" s="11"/>
+      <c r="A27" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="15"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="15"/>
+      <c r="Q27" s="15"/>
+      <c r="R27" s="15"/>
+      <c r="S27" s="15"/>
+      <c r="T27" s="15"/>
+      <c r="U27" s="15"/>
+      <c r="V27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
-      <c r="O28" s="11"/>
-      <c r="P28" s="11"/>
-      <c r="Q28" s="11"/>
-      <c r="R28" s="11"/>
-      <c r="S28" s="11"/>
-      <c r="T28" s="11"/>
-      <c r="U28" s="11"/>
-      <c r="V28" s="11"/>
+      <c r="A28" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="15"/>
+      <c r="Q28" s="15"/>
+      <c r="R28" s="15"/>
+      <c r="S28" s="15"/>
+      <c r="T28" s="15"/>
+      <c r="U28" s="15"/>
+      <c r="V28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
-      <c r="O29" s="11"/>
-      <c r="P29" s="11"/>
-      <c r="Q29" s="11"/>
-      <c r="R29" s="11"/>
-      <c r="S29" s="11"/>
-      <c r="T29" s="11"/>
-      <c r="U29" s="11"/>
-      <c r="V29" s="11"/>
+      <c r="A29" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="11"/>
-      <c r="O30" s="11"/>
-      <c r="P30" s="11"/>
-      <c r="Q30" s="11"/>
-      <c r="R30" s="11"/>
-      <c r="S30" s="11"/>
-      <c r="T30" s="11"/>
-      <c r="U30" s="11"/>
-      <c r="V30" s="11"/>
+      <c r="A30" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="15"/>
+      <c r="M30" s="15"/>
+      <c r="N30" s="15"/>
+      <c r="O30" s="15"/>
+      <c r="P30" s="15"/>
+      <c r="Q30" s="15"/>
+      <c r="R30" s="15"/>
+      <c r="S30" s="15"/>
+      <c r="T30" s="15"/>
+      <c r="U30" s="15"/>
+      <c r="V30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
-      <c r="O31" s="11"/>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
-      <c r="T31" s="11"/>
-      <c r="U31" s="11"/>
-      <c r="V31" s="11"/>
+      <c r="A31" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="15"/>
+      <c r="Q31" s="15"/>
+      <c r="R31" s="15"/>
+      <c r="S31" s="15"/>
+      <c r="T31" s="15"/>
+      <c r="U31" s="15"/>
+      <c r="V31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
-      <c r="O32" s="11"/>
-      <c r="P32" s="11"/>
-      <c r="Q32" s="11"/>
-      <c r="R32" s="11"/>
-      <c r="S32" s="11"/>
-      <c r="T32" s="11"/>
-      <c r="U32" s="11"/>
-      <c r="V32" s="11"/>
+      <c r="A32" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="15"/>
+      <c r="P32" s="15"/>
+      <c r="Q32" s="15"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="15"/>
+      <c r="T32" s="15"/>
+      <c r="U32" s="15"/>
+      <c r="V32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
-      <c r="O33" s="11"/>
-      <c r="P33" s="11"/>
-      <c r="Q33" s="11"/>
-      <c r="R33" s="11"/>
-      <c r="S33" s="11"/>
-      <c r="T33" s="11"/>
-      <c r="U33" s="11"/>
-      <c r="V33" s="11"/>
+      <c r="A33" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15"/>
+      <c r="M33" s="15"/>
+      <c r="N33" s="15"/>
+      <c r="O33" s="15"/>
+      <c r="P33" s="15"/>
+      <c r="Q33" s="15"/>
+      <c r="R33" s="15"/>
+      <c r="S33" s="15"/>
+      <c r="T33" s="15"/>
+      <c r="U33" s="15"/>
+      <c r="V33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11"/>
-      <c r="O34" s="11"/>
-      <c r="P34" s="11"/>
-      <c r="Q34" s="11"/>
-      <c r="R34" s="11"/>
-      <c r="S34" s="11"/>
-      <c r="T34" s="11"/>
-      <c r="U34" s="11"/>
-      <c r="V34" s="11"/>
+      <c r="A34" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+      <c r="O34" s="15"/>
+      <c r="P34" s="15"/>
+      <c r="Q34" s="15"/>
+      <c r="R34" s="15"/>
+      <c r="S34" s="15"/>
+      <c r="T34" s="15"/>
+      <c r="U34" s="15"/>
+      <c r="V34" s="15"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -2806,7 +3178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2819,19 +3191,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2839,16 +3211,16 @@
         <v>22</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2856,16 +3228,16 @@
         <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>178</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2873,10 +3245,10 @@
         <v>24</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>179</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>